<commit_message>
Résolution des conflits 7c08962e040a97426f5b98786b53173233e02fdb
</commit_message>
<xml_diff>
--- a/htr-FHIR/ig/StructureDefinition-fr-informant-extension.xlsx
+++ b/htr-FHIR/ig/StructureDefinition-fr-informant-extension.xlsx
@@ -54,7 +54,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-03-10T13:00:25+00:00</t>
+    <t>2025-03-11T15:29:00+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -642,7 +642,7 @@
     <t>valueReference</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-practitionerRole-document)
+    <t xml:space="preserve">Reference(https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-practitionerRole-document|https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-related-person-document|https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-patient-fhir-document)
 </t>
   </si>
   <si>

</xml_diff>